<commit_message>
Removing unnecessary static table, update QA files to have correct file paths, updating EPA loading and cleaning steps to use monthly version when running eGRID at the annual level
</commit_message>
<xml_diff>
--- a/data/1_production_model/static_tables/manual_corrections.xlsx
+++ b/data/1_production_model/static_tables/manual_corrections.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\projects\eGrid\production_model\users\gofortht\data\static_tables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\projects\eGrid\production_model\users\gofortht\data\1_production_model\static_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{053205CE-D372-4165-AD7C-5ECADBBADABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3023DB3-B30F-482D-8EFE-9F67B839FF96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" firstSheet="1" activeTab="3" xr2:uid="{FA61C6A3-A5F8-4301-A228-D222830EB6CC}"/>
+    <workbookView xWindow="9585" yWindow="1740" windowWidth="14595" windowHeight="11250" activeTab="3" xr2:uid="{FA61C6A3-A5F8-4301-A228-D222830EB6CC}"/>
   </bookViews>
   <sheets>
     <sheet name="epa_clean" sheetId="5" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="60">
   <si>
     <t>plant_id</t>
   </si>
@@ -205,6 +205,21 @@
   </si>
   <si>
     <t>MECCU2</t>
+  </si>
+  <si>
+    <t>61082</t>
+  </si>
+  <si>
+    <t>DL</t>
+  </si>
+  <si>
+    <t>so2_controls</t>
+  </si>
+  <si>
+    <t>nox_controls</t>
+  </si>
+  <si>
+    <t>SNCR</t>
   </si>
 </sst>
 </file>
@@ -823,7 +838,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C1A8242-D17A-4DAB-8319-EC8C1026D049}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="8.140625" style="3" bestFit="1" customWidth="1"/>
@@ -1169,6 +1184,28 @@
       </c>
       <c r="E24" s="3" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" t="s">
+        <v>58</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding 2024 manual corrections
</commit_message>
<xml_diff>
--- a/data/1_production_model/static_tables/manual_corrections.xlsx
+++ b/data/1_production_model/static_tables/manual_corrections.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\projects\eGrid\production_model\users\gofortht\data\1_production_model\static_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3023DB3-B30F-482D-8EFE-9F67B839FF96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9B1683D-9804-49E1-9C4C-FA202F083A87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9585" yWindow="1740" windowWidth="14595" windowHeight="11250" activeTab="3" xr2:uid="{FA61C6A3-A5F8-4301-A228-D222830EB6CC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{FA61C6A3-A5F8-4301-A228-D222830EB6CC}"/>
   </bookViews>
   <sheets>
     <sheet name="epa_clean" sheetId="5" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="61">
   <si>
     <t>plant_id</t>
   </si>
@@ -183,9 +183,6 @@
     <t>52193</t>
   </si>
   <si>
-    <t>21H</t>
-  </si>
-  <si>
     <t>21H701</t>
   </si>
   <si>
@@ -220,6 +217,12 @@
   </si>
   <si>
     <t>SNCR</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>21H1</t>
   </si>
 </sst>
 </file>
@@ -611,44 +614,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D934C9D8-7DA6-4C13-BBA3-1B260AEBF0C8}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
+        <v>2024</v>
+      </c>
+      <c r="B2">
         <v>880004</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>0</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>57788</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
+        <v>2023</v>
+      </c>
+      <c r="B3">
         <v>10154</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>37</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>38</v>
       </c>
     </row>
@@ -659,33 +671,39 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD042B8F-EA7C-4084-B7F4-709825082C60}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
+        <v>2024</v>
+      </c>
+      <c r="B2">
         <v>60910</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>40</v>
       </c>
     </row>
@@ -697,139 +715,163 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{791B152A-9A17-4C98-BF21-937C78FED9AB}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="18.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
+        <v>2024</v>
+      </c>
+      <c r="B2">
         <v>7512</v>
       </c>
-      <c r="B2" s="3">
+      <c r="C2" s="3">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
+        <v>2024</v>
+      </c>
+      <c r="B3">
         <v>7512</v>
       </c>
-      <c r="B3" s="3">
+      <c r="C3" s="3">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
+        <v>2024</v>
+      </c>
+      <c r="B4">
         <v>7512</v>
       </c>
-      <c r="B4" s="3">
+      <c r="C4" s="3">
         <v>3</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5">
         <v>664</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
+        <v>2024</v>
+      </c>
+      <c r="B6">
         <v>56032</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="B7">
         <v>55350</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
+        <v>2023</v>
+      </c>
+      <c r="B8">
         <v>55350</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B11"/>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C11"/>
-      <c r="E11"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B12"/>
+      <c r="D11"/>
+      <c r="F11"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C12"/>
-      <c r="E12"/>
+      <c r="D12"/>
+      <c r="F12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -838,374 +880,452 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C1A8242-D17A-4DAB-8319-EC8C1026D049}">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="8.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="8.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.85546875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2024</v>
+      </c>
+      <c r="B2" s="3">
         <v>55248</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="3">
+      <c r="F2" s="3">
         <v>2847</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2024</v>
+      </c>
+      <c r="B3" s="3">
         <v>2847</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2024</v>
+      </c>
+      <c r="B4" s="3">
         <v>2707</v>
       </c>
-      <c r="B4" s="3">
+      <c r="C4" s="3">
         <v>1</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5" s="3">
         <v>2707</v>
       </c>
-      <c r="B5" s="3">
+      <c r="C5" s="3">
         <v>2</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2024</v>
+      </c>
+      <c r="B6" s="3">
         <v>2707</v>
       </c>
-      <c r="B6" s="3">
+      <c r="C6" s="3">
         <v>3</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2024</v>
+      </c>
+      <c r="B7" s="3">
         <v>2707</v>
       </c>
-      <c r="B7" s="3">
+      <c r="C7" s="3">
         <v>4</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>1</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2023</v>
+      </c>
+      <c r="B8" s="3">
         <v>7832</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2023</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2023</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2024</v>
+      </c>
+      <c r="B11" s="3">
         <v>7063</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>19</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2024</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2024</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2024</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="C14" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>2024</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="F15" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>2024</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>2024</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="C17" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>31</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="F17" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>2024</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="C18" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>30</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="F18" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>2024</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" t="s">
+        <v>50</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>2024</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D20" t="s">
         <v>36</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E20" t="s">
+        <v>50</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E19" s="3" t="s">
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>2024</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>2024</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C22" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" t="s">
+        <v>50</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>2024</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+      <c r="D23" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>2024</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" t="s">
-        <v>51</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B22" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" t="s">
-        <v>51</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="C24" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D24" t="s">
         <v>13</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E24" t="s">
         <v>12</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="F24" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B24" s="3" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>2024</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" t="s">
-        <v>12</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+      <c r="E25" t="s">
+        <v>56</v>
+      </c>
+      <c r="F25" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D25" t="s">
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>2024</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E26" t="s">
         <v>57</v>
       </c>
-      <c r="E25" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D26" t="s">
+      <c r="F26" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1216,96 +1336,99 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A26772A-0AAB-4516-99B5-5272EE829F50}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" style="3"/>
-    <col min="2" max="2" width="19.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" style="3"/>
+    <col min="3" max="3" width="19.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B2" s="3">
         <v>54975</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>32.380032</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="3">
         <v>62262</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>42.899028999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B4" s="3">
         <v>54975</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>-106.753716</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="3">
         <v>62262</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>-75.458455999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>42.502749999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>-79.281723</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Adding plant to EPA plants to delete, removing duplicate EF, adding primary fuel correction to manual_corrections file, re-ordering monthly and annual generator/unit file creation to output both annual and monthly versions when running annual temporal res due to plant file dependencies, updating QA all
</commit_message>
<xml_diff>
--- a/data/1_production_model/static_tables/manual_corrections.xlsx
+++ b/data/1_production_model/static_tables/manual_corrections.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\projects\eGrid\production_model\users\gofortht\data\1_production_model\static_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9B1683D-9804-49E1-9C4C-FA202F083A87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7DE75F5-AD3E-4299-A41C-41B645F32D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{FA61C6A3-A5F8-4301-A228-D222830EB6CC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{FA61C6A3-A5F8-4301-A228-D222830EB6CC}"/>
   </bookViews>
   <sheets>
     <sheet name="epa_clean" sheetId="5" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="72">
   <si>
     <t>plant_id</t>
   </si>
@@ -223,6 +223,39 @@
   </si>
   <si>
     <t>21H1</t>
+  </si>
+  <si>
+    <t>57025</t>
+  </si>
+  <si>
+    <t>GEN1</t>
+  </si>
+  <si>
+    <t>GEN2</t>
+  </si>
+  <si>
+    <t>GEN3</t>
+  </si>
+  <si>
+    <t>GEN4</t>
+  </si>
+  <si>
+    <t>GEN5</t>
+  </si>
+  <si>
+    <t>IC</t>
+  </si>
+  <si>
+    <t>NG</t>
+  </si>
+  <si>
+    <t>50932</t>
+  </si>
+  <si>
+    <t>72-04</t>
+  </si>
+  <si>
+    <t>72-05</t>
   </si>
 </sst>
 </file>
@@ -880,7 +913,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C1A8242-D17A-4DAB-8319-EC8C1026D049}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="8.140625" style="3" bestFit="1" customWidth="1"/>
@@ -1326,6 +1359,146 @@
       </c>
       <c r="F26" s="3" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>2024</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D27" t="s">
+        <v>67</v>
+      </c>
+      <c r="E27" t="s">
+        <v>50</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>2024</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D28" t="s">
+        <v>67</v>
+      </c>
+      <c r="E28" t="s">
+        <v>50</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>2024</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" t="s">
+        <v>67</v>
+      </c>
+      <c r="E29" t="s">
+        <v>50</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>2024</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D30" t="s">
+        <v>67</v>
+      </c>
+      <c r="E30" t="s">
+        <v>50</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>2024</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D31" t="s">
+        <v>67</v>
+      </c>
+      <c r="E31" t="s">
+        <v>50</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>2024</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D32" t="s">
+        <v>67</v>
+      </c>
+      <c r="E32" t="s">
+        <v>50</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>2024</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D33" t="s">
+        <v>67</v>
+      </c>
+      <c r="E33" t="s">
+        <v>50</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>